<commit_message>
docs: sync tuner guardrails and canonical requirements
</commit_message>
<xml_diff>
--- a/00_Documentation/requirements/user-stories-v1.xlsx
+++ b/00_Documentation/requirements/user-stories-v1.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Estudio y Personales\SENA\01 Software Development and Analysis\02_Planning\03_Assessments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Estudio y Personales\SENA\01 Software Development and Analysis\MusicAI\00_Documentation\requirements\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A0062782-D1F7-478A-AF85-26E86434BCCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8742CB92-A668-415D-95BA-CAA15A80D6C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="861" xr2:uid="{89B37B4C-B566-4606-BA64-38B82CB154B8}"/>
   </bookViews>
@@ -3969,45 +3969,6 @@
     <t>HISTORIAS DE USUARIO - PANTALLA AFINADOR</t>
   </si>
   <si>
-    <t>Afinar una cuerda de la guitarra mediante el micrófono del dispositivo</t>
-  </si>
-  <si>
-    <t>Ajustar la cuerda seleccionada hasta alcanzar la nota objetivo correspondiente a la afinación configurada</t>
-  </si>
-  <si>
-    <t>1. El estudiante debe poder acceder al Afinador desde la navegación principal de MusicAI.
-2. El sistema debe solicitar autorización para utilizar el micrófono cuando sea necesario.
-3. El estudiante debe poder seleccionar manualmente la cuerda que desea afinar.
-4. El sistema debe analizar mediante el micrófono la frecuencia del sonido producido por la cuerda.
-5. El sistema debe identificar la nota detectada y compararla con la nota objetivo de la cuerda seleccionada.
-6. El sistema debe indicar la desviación de afinación en cents.
-7. El sistema debe informar si la cuerda debe subir de afinación, bajar de afinación o se encuentra afinada.
-8. La información debe actualizarse mientras el estudiante continúe produciendo sonido.
-9. Si no existe una señal suficientemente válida para realizar la medición, el sistema debe indicarlo sin presentar una afinación incorrecta como válida.
-10. El audio utilizado para la detección debe procesarse únicamente para la afinación y no almacenarse permanentemente.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Objetivo:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Validar que el estudiante pueda seleccionar una cuerda y afinarla utilizando detección cromática mediante el micrófono del dispositivo.</t>
-    </r>
-  </si>
-  <si>
     <r>
       <rPr>
         <b/>
@@ -4029,61 +3990,6 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">Nombre Requerimiento: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>R39 – Afinación cromática de guitarra</t>
-    </r>
-  </si>
-  <si>
-    <t>1. El estudiante debe tener una sesión autenticada.
-2. El dispositivo debe disponer de micrófono compatible.
-3. El permiso de micrófono debe estar disponible.
-4. Debe existir una afinación objetivo seleccionada.</t>
-  </si>
-  <si>
-    <t>1. El estudiante selecciona una cuerda.
-2. El sistema detecta la frecuencia y nota producidas.
-3. Se muestra la desviación respecto a la nota objetivo.
-4. El estudiante recibe una indicación clara para subir, bajar o mantener la afinación.
-5. El audio no queda almacenado.</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t>Relación de navegación:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <color theme="1"/>
-        <rFont val="Arial"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve"> Pantallas con navegación principal → Afinador - Afinador → Pantallas con navegación principal</t>
-    </r>
-  </si>
-  <si>
     <t>R40 – Seleccionar la afinación de la guitarra</t>
   </si>
   <si>
@@ -4091,14 +3997,6 @@
   </si>
   <si>
     <t>Utilizar las notas objetivo correspondientes a la afinación que desea aplicar al instrumento</t>
-  </si>
-  <si>
-    <t>1. El Afinador debe permitir seleccionar una afinación entre las disponibles para el MVP.
-2. El sistema debe ofrecer las afinaciones E Standard, Eb Standard, D Standard, Drop D, C Standard y Drop C.
-3. Al seleccionar una afinación, el sistema debe actualizar las notas objetivo de las seis cuerdas.
-4. La cuerda seleccionada para afinar debe utilizar como referencia la nota correspondiente al preset activo.
-5. Cambiar la afinación no debe modificar progreso académico, XP, racha ni resultados del estudiante.
-6. La afinación seleccionada debe permanecer activa mientras el estudiante utilice el Afinador o hasta que seleccione otra disponible.</t>
   </si>
   <si>
     <r>
@@ -4725,6 +4623,119 @@
   </si>
   <si>
     <t>R39 – Afinar una cuerda de la guitarra</t>
+  </si>
+  <si>
+    <t>Afinar una cuerda de la guitarra mediante el micrófono del dispositivo, permitiendo que MusicAI identifique automáticamente la cuerda pulsada.</t>
+  </si>
+  <si>
+    <t>Ajustar la cuerda detectada hasta alcanzar la nota objetivo correspondiente a la afinación predefinida activa.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Objetivo:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Validar que el estudiante pueda afinar las cuerdas de su guitarra permitiendo que MusicAI identifique automáticamente la cuerda pulsada, muestre su nota objetivo y proporcione retroalimentación visual clara sobre su desviación de afinación.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">Nombre Requerimiento: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>R39 – Afinación automática de cuerdas de guitarra</t>
+    </r>
+  </si>
+  <si>
+    <t>1. El estudiante debe tener una sesión autenticada.
+2. El dispositivo debe disponer de un micrófono compatible.
+3. El permiso de micrófono debe estar disponible cuando la implementación real lo requiera.
+4. Debe existir una afinación predefinida activa que establezca las notas objetivo de las seis cuerdas.
+5. El sistema debe disponer de las notas y frecuencias objetivo correspondientes a la afinación activa.</t>
+  </si>
+  <si>
+    <t>1. El estudiante pulsa una cuerda de la guitarra sin seleccionarla previamente en la interfaz.
+2. MusicAI identifica automáticamente la cuerda correspondiente.
+3. El sistema muestra la nota objetivo y su frecuencia de referencia.
+4. El sistema detecta la frecuencia y la nota producidas.
+5. El estudiante visualiza la desviación respecto a la nota objetivo mediante un indicador intuitivo de grave, agudo o afinado.
+6. La cuerda detectada se destaca visualmente mientras está siendo afinada.
+7. Cuando la cuerda alcanza la afinación correcta, queda identificada visualmente como afinada.
+8. Al pulsar otra cuerda, el sistema cambia automáticamente el contexto de afinación a la nueva cuerda detectada.
+9. El audio utilizado para la detección no queda almacenado permanentemente.
+10. El estudiante puede cerrar el Afinador y regresar al contexto anterior.</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Relación de navegación:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> Pantallas autenticadas con acceso al Afinador → Afinador → Contexto autenticado anterior</t>
+    </r>
+  </si>
+  <si>
+    <t>1. El Afinador debe permitir seleccionar una afinación entre las disponibles para el MVP.
+2. El sistema debe ofrecer las afinaciones E Standard, Eb Standard, D Standard, Drop D, C Standard y Drop C.
+3. Al seleccionar una afinación, el sistema debe actualizar las notas objetivo de las seis cuerdas.
+4. La cuerda identificada automáticamente por R39 debe utilizar como referencia la nota correspondiente al preset activo.
+5. Cambiar la afinación no debe modificar progreso académico, XP, racha ni resultados del estudiante.
+6. La afinación seleccionada debe permanecer activa mientras el estudiante utilice el Afinador o hasta que seleccione otra disponible.</t>
+  </si>
+  <si>
+    <t>1. El estudiante debe poder acceder al Afinador desde el entorno autenticado de MusicAI cuando necesite comprobar o corregir la afinación de su guitarra.
+2. El sistema debe solicitar autorización para utilizar el micrófono cuando sea necesario para realizar la afinación.
+3. El estudiante debe poder pulsar directamente una cuerda de la guitarra sin seleccionarla previamente en la interfaz.
+4. El sistema debe analizar mediante el micrófono la frecuencia y la nota producidas por la cuerda pulsada.
+5. El sistema debe identificar automáticamente la cuerda correspondiente a partir de la señal detectada y de la afinación predefinida activa.
+6. El sistema debe comparar la frecuencia y la nota detectadas con la frecuencia y la nota objetivo correspondientes a la cuerda identificada.
+7. El sistema debe mostrar de forma clara la nota objetivo y la frecuencia de referencia correspondiente a la cuerda identificada.
+8. El sistema debe indicar visualmente la desviación de afinación y permitir reconocer si el sonido se encuentra hacia una frecuencia más grave, más aguda o dentro del estado afinado.
+9. La cuerda identificada debe distinguirse visualmente de las demás mientras está siendo afinada.
+10. Cuando una cuerda alcance correctamente su nota objetivo, el sistema debe marcarla visualmente como afinada.
+11. Al pulsar otra cuerda, el sistema debe identificarla automáticamente y actualizar el feedback de afinación correspondiente sin requerir una selección manual previa.
+12. La información debe actualizarse mientras el estudiante continúe produciendo una señal válida.
+13. Si no existe una señal suficientemente válida o identificable para realizar la medición, el sistema debe evitar presentar una afinación incorrecta como válida.
+14. El audio utilizado para la detección debe procesarse únicamente para la afinación y no almacenarse permanentemente.
+15. El estudiante debe poder cerrar o cancelar el Afinador y regresar al contexto autenticado desde el cual lo abrió.</t>
   </si>
 </sst>
 </file>
@@ -5263,9 +5274,6 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -5278,6 +5286,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -5287,8 +5298,8 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -6069,7 +6080,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R36</v>
       </c>
@@ -6083,11 +6094,11 @@
         <v>343</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>421</v>
+        <v>412</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -6096,7 +6107,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -6105,23 +6116,23 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
-        <v>422</v>
+        <v>413</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>344</v>
       </c>
@@ -6130,7 +6141,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>345</v>
       </c>
@@ -6139,24 +6150,24 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>423</v>
+        <v>414</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>424</v>
+        <v>415</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
-        <v>425</v>
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
+        <v>416</v>
       </c>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -6191,7 +6202,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="123" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R37</v>
       </c>
@@ -6209,7 +6220,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -6218,7 +6229,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -6227,14 +6238,14 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>350</v>
       </c>
@@ -6243,7 +6254,7 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>351</v>
       </c>
@@ -6252,7 +6263,7 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
         <v>352</v>
       </c>
@@ -6261,7 +6272,7 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
@@ -6276,8 +6287,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
         <v>355</v>
       </c>
       <c r="C25" s="48"/>
@@ -6313,7 +6324,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="179.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v>R38</v>
       </c>
@@ -6327,11 +6338,11 @@
         <v>358</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>426</v>
+        <v>417</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -6340,7 +6351,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -6349,23 +6360,23 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="63.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
-        <v>427</v>
+        <v>418</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
         <v>359</v>
       </c>
@@ -6374,7 +6385,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
         <v>360</v>
       </c>
@@ -6383,24 +6394,24 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>428</v>
+        <v>419</v>
       </c>
       <c r="D37" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>429</v>
+        <v>420</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
+      <c r="A38" s="52"/>
       <c r="B38" s="55" t="s">
-        <v>430</v>
+        <v>421</v>
       </c>
       <c r="C38" s="48"/>
       <c r="D38" s="48"/>
@@ -6432,10 +6443,10 @@
   <sheetFormatPr defaultColWidth="0" defaultRowHeight="0" customHeight="1" zeroHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="4.28515625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="46.42578125" style="17" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="42" style="17" customWidth="1"/>
+    <col min="2" max="2" width="54.140625" style="17" customWidth="1"/>
+    <col min="3" max="3" width="47.140625" style="17" customWidth="1"/>
     <col min="4" max="4" width="28.28515625" style="17" customWidth="1"/>
-    <col min="5" max="5" width="94.140625" style="17" customWidth="1"/>
+    <col min="5" max="5" width="105.42578125" style="17" customWidth="1"/>
     <col min="6" max="6" width="11" style="1" customWidth="1"/>
     <col min="7" max="16384" width="11" style="1" hidden="1"/>
   </cols>
@@ -6451,7 +6462,7 @@
     </row>
     <row r="2" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="44" t="s">
-        <v>431</v>
+        <v>422</v>
       </c>
       <c r="B2" s="45"/>
       <c r="C2" s="45"/>
@@ -6475,8 +6486,8 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="165.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+    <row r="4" spans="1:5" ht="294" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R39</v>
       </c>
@@ -6484,17 +6495,17 @@
         <v>46</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>366</v>
+        <v>423</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>367</v>
+        <v>424</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>368</v>
+        <v>431</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -6503,7 +6514,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -6512,58 +6523,58 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
-    <row r="8" spans="1:5" ht="55.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+    <row r="8" spans="1:5" ht="63.75" x14ac:dyDescent="0.2">
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
-        <v>369</v>
+        <v>425</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
-        <v>370</v>
+        <v>366</v>
       </c>
       <c r="C9" s="10"/>
       <c r="D9" s="10"/>
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
-        <v>371</v>
+        <v>426</v>
       </c>
       <c r="C10" s="24"/>
       <c r="D10" s="24"/>
       <c r="E10" s="25"/>
     </row>
-    <row r="11" spans="1:5" ht="102.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+    <row r="11" spans="1:5" ht="141" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>372</v>
+        <v>427</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>373</v>
+        <v>428</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
+      <c r="A12" s="52"/>
       <c r="B12" s="55" t="s">
-        <v>374</v>
+        <v>429</v>
       </c>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -6573,7 +6584,7 @@
     <row r="14" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="44" t="s">
-        <v>375</v>
+        <v>367</v>
       </c>
       <c r="B15" s="45"/>
       <c r="C15" s="45"/>
@@ -6598,7 +6609,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="120.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R40</v>
       </c>
@@ -6606,17 +6617,17 @@
         <v>46</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>376</v>
+        <v>368</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>377</v>
+        <v>369</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>378</v>
+        <v>430</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -6625,7 +6636,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -6634,58 +6645,58 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
-    <row r="21" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+    <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
-        <v>379</v>
+        <v>370</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="C22" s="10"/>
       <c r="D22" s="10"/>
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
-        <v>381</v>
+        <v>372</v>
       </c>
       <c r="C23" s="24"/>
       <c r="D23" s="24"/>
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>382</v>
+        <v>373</v>
       </c>
       <c r="D24" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>383</v>
+        <v>374</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
-        <v>384</v>
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
+        <v>375</v>
       </c>
       <c r="C25" s="48"/>
       <c r="D25" s="48"/>
@@ -6756,7 +6767,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v/>
       </c>
@@ -6768,7 +6779,7 @@
       <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -6777,7 +6788,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -6786,14 +6797,14 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
         <v>361</v>
       </c>
@@ -6802,7 +6813,7 @@
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="36" t="s">
         <v>362</v>
       </c>
@@ -6811,7 +6822,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="37" t="s">
         <v>363</v>
       </c>
@@ -6820,7 +6831,7 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
@@ -6831,8 +6842,8 @@
       <c r="E11" s="21"/>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
         <v>364</v>
       </c>
       <c r="C12" s="48"/>
@@ -6866,7 +6877,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v/>
       </c>
@@ -6878,7 +6889,7 @@
       <c r="E17" s="7"/>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -6887,7 +6898,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -6896,14 +6907,14 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>361</v>
       </c>
@@ -6912,7 +6923,7 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="36" t="s">
         <v>362</v>
       </c>
@@ -6921,7 +6932,7 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="37" t="s">
         <v>363</v>
       </c>
@@ -6930,7 +6941,7 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
@@ -6941,8 +6952,8 @@
       <c r="E24" s="21"/>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
         <v>364</v>
       </c>
       <c r="C25" s="48"/>
@@ -6976,7 +6987,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v/>
       </c>
@@ -6988,7 +6999,7 @@
       <c r="E30" s="7"/>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -6997,7 +7008,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -7006,14 +7017,14 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
         <v>361</v>
       </c>
@@ -7022,7 +7033,7 @@
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="36" t="s">
         <v>362</v>
       </c>
@@ -7031,7 +7042,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="37" t="s">
         <v>363</v>
       </c>
@@ -7040,7 +7051,7 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
@@ -7051,8 +7062,8 @@
       <c r="E37" s="21"/>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>364</v>
       </c>
       <c r="C38" s="48"/>
@@ -7086,7 +7097,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="51" t="str">
+      <c r="A43" s="50" t="str">
         <f>LEFT(A41,3)</f>
         <v/>
       </c>
@@ -7098,7 +7109,7 @@
       <c r="E43" s="7"/>
     </row>
     <row r="44" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="52"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="23"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -7107,7 +7118,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="52"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="29" t="s">
         <v>8</v>
       </c>
@@ -7116,14 +7127,14 @@
       <c r="E45" s="11"/>
     </row>
     <row r="46" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A46" s="52"/>
+      <c r="A46" s="51"/>
       <c r="B46" s="22"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="11"/>
     </row>
     <row r="47" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A47" s="52"/>
+      <c r="A47" s="51"/>
       <c r="B47" s="26" t="s">
         <v>361</v>
       </c>
@@ -7132,7 +7143,7 @@
       <c r="E47" s="11"/>
     </row>
     <row r="48" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A48" s="52"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="36" t="s">
         <v>362</v>
       </c>
@@ -7141,7 +7152,7 @@
       <c r="E48" s="11"/>
     </row>
     <row r="49" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="52"/>
+      <c r="A49" s="51"/>
       <c r="B49" s="37" t="s">
         <v>363</v>
       </c>
@@ -7150,7 +7161,7 @@
       <c r="E49" s="25"/>
     </row>
     <row r="50" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="52"/>
+      <c r="A50" s="51"/>
       <c r="B50" s="18" t="s">
         <v>6</v>
       </c>
@@ -7161,8 +7172,8 @@
       <c r="E50" s="21"/>
     </row>
     <row r="51" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="53"/>
-      <c r="B51" s="54" t="s">
+      <c r="A51" s="52"/>
+      <c r="B51" s="53" t="s">
         <v>364</v>
       </c>
       <c r="C51" s="48"/>
@@ -7196,7 +7207,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="51" t="str">
+      <c r="A56" s="50" t="str">
         <f>LEFT(A54,3)</f>
         <v/>
       </c>
@@ -7208,7 +7219,7 @@
       <c r="E56" s="7"/>
     </row>
     <row r="57" spans="1:5" ht="13.5" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="52"/>
+      <c r="A57" s="51"/>
       <c r="B57" s="23"/>
       <c r="C57" s="8"/>
       <c r="D57" s="8"/>
@@ -7217,7 +7228,7 @@
       </c>
     </row>
     <row r="58" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="52"/>
+      <c r="A58" s="51"/>
       <c r="B58" s="29" t="s">
         <v>8</v>
       </c>
@@ -7226,14 +7237,14 @@
       <c r="E58" s="11"/>
     </row>
     <row r="59" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A59" s="52"/>
+      <c r="A59" s="51"/>
       <c r="B59" s="22"/>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="11"/>
     </row>
     <row r="60" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A60" s="52"/>
+      <c r="A60" s="51"/>
       <c r="B60" s="26" t="s">
         <v>361</v>
       </c>
@@ -7242,7 +7253,7 @@
       <c r="E60" s="11"/>
     </row>
     <row r="61" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A61" s="52"/>
+      <c r="A61" s="51"/>
       <c r="B61" s="36" t="s">
         <v>362</v>
       </c>
@@ -7251,7 +7262,7 @@
       <c r="E61" s="11"/>
     </row>
     <row r="62" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="52"/>
+      <c r="A62" s="51"/>
       <c r="B62" s="37" t="s">
         <v>363</v>
       </c>
@@ -7260,7 +7271,7 @@
       <c r="E62" s="25"/>
     </row>
     <row r="63" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="52"/>
+      <c r="A63" s="51"/>
       <c r="B63" s="18" t="s">
         <v>6</v>
       </c>
@@ -7271,8 +7282,8 @@
       <c r="E63" s="21"/>
     </row>
     <row r="64" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="53"/>
-      <c r="B64" s="54" t="s">
+      <c r="A64" s="52"/>
+      <c r="B64" s="53" t="s">
         <v>364</v>
       </c>
       <c r="C64" s="48"/>
@@ -7306,7 +7317,7 @@
       </c>
     </row>
     <row r="69" spans="1:5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="51" t="str">
+      <c r="A69" s="50" t="str">
         <f>LEFT(A67,3)</f>
         <v/>
       </c>
@@ -7318,7 +7329,7 @@
       <c r="E69" s="7"/>
     </row>
     <row r="70" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="52"/>
+      <c r="A70" s="51"/>
       <c r="B70" s="23"/>
       <c r="C70" s="8"/>
       <c r="D70" s="8"/>
@@ -7327,7 +7338,7 @@
       </c>
     </row>
     <row r="71" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="52"/>
+      <c r="A71" s="51"/>
       <c r="B71" s="29" t="s">
         <v>8</v>
       </c>
@@ -7336,14 +7347,14 @@
       <c r="E71" s="11"/>
     </row>
     <row r="72" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="52"/>
+      <c r="A72" s="51"/>
       <c r="B72" s="22"/>
       <c r="C72" s="10"/>
       <c r="D72" s="10"/>
       <c r="E72" s="11"/>
     </row>
     <row r="73" spans="1:5" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A73" s="52"/>
+      <c r="A73" s="51"/>
       <c r="B73" s="26" t="s">
         <v>361</v>
       </c>
@@ -7352,7 +7363,7 @@
       <c r="E73" s="11"/>
     </row>
     <row r="74" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="52"/>
+      <c r="A74" s="51"/>
       <c r="B74" s="36" t="s">
         <v>362</v>
       </c>
@@ -7361,7 +7372,7 @@
       <c r="E74" s="11"/>
     </row>
     <row r="75" spans="1:5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="52"/>
+      <c r="A75" s="51"/>
       <c r="B75" s="37" t="s">
         <v>363</v>
       </c>
@@ -7370,7 +7381,7 @@
       <c r="E75" s="25"/>
     </row>
     <row r="76" spans="1:5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="52"/>
+      <c r="A76" s="51"/>
       <c r="B76" s="18" t="s">
         <v>6</v>
       </c>
@@ -7381,8 +7392,8 @@
       <c r="E76" s="21"/>
     </row>
     <row r="77" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="53"/>
-      <c r="B77" s="54" t="s">
+      <c r="A77" s="52"/>
+      <c r="B77" s="53" t="s">
         <v>364</v>
       </c>
       <c r="C77" s="48"/>
@@ -7416,7 +7427,7 @@
       </c>
     </row>
     <row r="82" spans="1:5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="51" t="str">
+      <c r="A82" s="50" t="str">
         <f>LEFT(A80,3)</f>
         <v/>
       </c>
@@ -7428,7 +7439,7 @@
       <c r="E82" s="7"/>
     </row>
     <row r="83" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="52"/>
+      <c r="A83" s="51"/>
       <c r="B83" s="23"/>
       <c r="C83" s="8"/>
       <c r="D83" s="8"/>
@@ -7437,7 +7448,7 @@
       </c>
     </row>
     <row r="84" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="52"/>
+      <c r="A84" s="51"/>
       <c r="B84" s="29" t="s">
         <v>8</v>
       </c>
@@ -7446,14 +7457,14 @@
       <c r="E84" s="11"/>
     </row>
     <row r="85" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="52"/>
+      <c r="A85" s="51"/>
       <c r="B85" s="22"/>
       <c r="C85" s="10"/>
       <c r="D85" s="10"/>
       <c r="E85" s="11"/>
     </row>
     <row r="86" spans="1:5" customFormat="1" ht="15" x14ac:dyDescent="0.25">
-      <c r="A86" s="52"/>
+      <c r="A86" s="51"/>
       <c r="B86" s="26" t="s">
         <v>361</v>
       </c>
@@ -7462,7 +7473,7 @@
       <c r="E86" s="11"/>
     </row>
     <row r="87" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="52"/>
+      <c r="A87" s="51"/>
       <c r="B87" s="36" t="s">
         <v>362</v>
       </c>
@@ -7471,7 +7482,7 @@
       <c r="E87" s="11"/>
     </row>
     <row r="88" spans="1:5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="52"/>
+      <c r="A88" s="51"/>
       <c r="B88" s="37" t="s">
         <v>363</v>
       </c>
@@ -7480,7 +7491,7 @@
       <c r="E88" s="25"/>
     </row>
     <row r="89" spans="1:5" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="52"/>
+      <c r="A89" s="51"/>
       <c r="B89" s="18" t="s">
         <v>6</v>
       </c>
@@ -7491,8 +7502,8 @@
       <c r="E89" s="21"/>
     </row>
     <row r="90" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="53"/>
-      <c r="B90" s="54" t="s">
+      <c r="A90" s="52"/>
+      <c r="B90" s="53" t="s">
         <v>364</v>
       </c>
       <c r="C90" s="48"/>
@@ -7503,19 +7514,6 @@
     <row r="92" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A17:A25"/>
-    <mergeCell ref="B25:E25"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:A12"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="A15:E15"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A30:A38"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A43:A51"/>
-    <mergeCell ref="B51:E51"/>
     <mergeCell ref="A80:E80"/>
     <mergeCell ref="A82:A90"/>
     <mergeCell ref="B90:E90"/>
@@ -7525,6 +7523,19 @@
     <mergeCell ref="A67:E67"/>
     <mergeCell ref="A69:A77"/>
     <mergeCell ref="B77:E77"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A30:A38"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A43:A51"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="A17:A25"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:A12"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A15:E15"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -7664,7 +7675,7 @@
     </row>
     <row r="12" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A12" s="40"/>
-      <c r="B12" s="50" t="s">
+      <c r="B12" s="58" t="s">
         <v>77</v>
       </c>
       <c r="C12" s="48"/>
@@ -7837,7 +7848,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="128.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="s">
+      <c r="A30" s="50" t="s">
         <v>53</v>
       </c>
       <c r="B30" s="5" t="s">
@@ -7854,14 +7865,14 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
       <c r="E31" s="9"/>
     </row>
     <row r="32" spans="1:5" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -7870,14 +7881,14 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
         <v>89</v>
       </c>
@@ -7886,7 +7897,7 @@
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
         <v>67</v>
       </c>
@@ -7895,7 +7906,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
         <v>90</v>
       </c>
@@ -7904,7 +7915,7 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
@@ -7919,8 +7930,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>54</v>
       </c>
       <c r="C38" s="48"/>
@@ -7956,7 +7967,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="51" t="s">
+      <c r="A43" s="50" t="s">
         <v>56</v>
       </c>
       <c r="B43" s="5" t="s">
@@ -7973,14 +7984,14 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="52"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="23"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
       <c r="E44" s="9"/>
     </row>
     <row r="45" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="52"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="29" t="s">
         <v>8</v>
       </c>
@@ -7989,14 +8000,14 @@
       <c r="E45" s="11"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="52"/>
+      <c r="A46" s="51"/>
       <c r="B46" s="22"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="11"/>
     </row>
     <row r="47" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A47" s="52"/>
+      <c r="A47" s="51"/>
       <c r="B47" s="26" t="s">
         <v>96</v>
       </c>
@@ -8005,7 +8016,7 @@
       <c r="E47" s="11"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="52"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="27" t="s">
         <v>57</v>
       </c>
@@ -8014,7 +8025,7 @@
       <c r="E48" s="11"/>
     </row>
     <row r="49" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="52"/>
+      <c r="A49" s="51"/>
       <c r="B49" s="28" t="s">
         <v>58</v>
       </c>
@@ -8023,7 +8034,7 @@
       <c r="E49" s="25"/>
     </row>
     <row r="50" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="52"/>
+      <c r="A50" s="51"/>
       <c r="B50" s="18" t="s">
         <v>6</v>
       </c>
@@ -8038,7 +8049,7 @@
       </c>
     </row>
     <row r="51" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="53"/>
+      <c r="A51" s="52"/>
       <c r="B51" s="55" t="s">
         <v>99</v>
       </c>
@@ -8075,7 +8086,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="51" t="s">
+      <c r="A56" s="50" t="s">
         <v>60</v>
       </c>
       <c r="B56" s="5" t="s">
@@ -8092,14 +8103,14 @@
       </c>
     </row>
     <row r="57" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="52"/>
+      <c r="A57" s="51"/>
       <c r="B57" s="23"/>
       <c r="C57" s="8"/>
       <c r="D57" s="8"/>
       <c r="E57" s="9"/>
     </row>
     <row r="58" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="52"/>
+      <c r="A58" s="51"/>
       <c r="B58" s="29" t="s">
         <v>8</v>
       </c>
@@ -8108,14 +8119,14 @@
       <c r="E58" s="11"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" s="52"/>
+      <c r="A59" s="51"/>
       <c r="B59" s="22"/>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="11"/>
     </row>
     <row r="60" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A60" s="52"/>
+      <c r="A60" s="51"/>
       <c r="B60" s="26" t="s">
         <v>102</v>
       </c>
@@ -8124,7 +8135,7 @@
       <c r="E60" s="11"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A61" s="52"/>
+      <c r="A61" s="51"/>
       <c r="B61" s="27" t="s">
         <v>63</v>
       </c>
@@ -8133,7 +8144,7 @@
       <c r="E61" s="11"/>
     </row>
     <row r="62" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="52"/>
+      <c r="A62" s="51"/>
       <c r="B62" s="28" t="s">
         <v>64</v>
       </c>
@@ -8142,7 +8153,7 @@
       <c r="E62" s="25"/>
     </row>
     <row r="63" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="52"/>
+      <c r="A63" s="51"/>
       <c r="B63" s="18" t="s">
         <v>6</v>
       </c>
@@ -8157,8 +8168,8 @@
       </c>
     </row>
     <row r="64" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="53"/>
-      <c r="B64" s="54" t="s">
+      <c r="A64" s="52"/>
+      <c r="B64" s="53" t="s">
         <v>65</v>
       </c>
       <c r="C64" s="48"/>
@@ -8194,7 +8205,7 @@
       </c>
     </row>
     <row r="69" spans="1:5" ht="115.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="51" t="str">
+      <c r="A69" s="50" t="str">
         <f>LEFT(A67,3)</f>
         <v>R09</v>
       </c>
@@ -8212,7 +8223,7 @@
       </c>
     </row>
     <row r="70" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="52"/>
+      <c r="A70" s="51"/>
       <c r="B70" s="23"/>
       <c r="C70" s="8"/>
       <c r="D70" s="8"/>
@@ -8221,7 +8232,7 @@
       </c>
     </row>
     <row r="71" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="52"/>
+      <c r="A71" s="51"/>
       <c r="B71" s="29" t="s">
         <v>8</v>
       </c>
@@ -8230,14 +8241,14 @@
       <c r="E71" s="11"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A72" s="52"/>
+      <c r="A72" s="51"/>
       <c r="B72" s="22"/>
       <c r="C72" s="10"/>
       <c r="D72" s="10"/>
       <c r="E72" s="11"/>
     </row>
     <row r="73" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A73" s="52"/>
+      <c r="A73" s="51"/>
       <c r="B73" s="26" t="s">
         <v>109</v>
       </c>
@@ -8246,7 +8257,7 @@
       <c r="E73" s="11"/>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A74" s="52"/>
+      <c r="A74" s="51"/>
       <c r="B74" s="27" t="s">
         <v>69</v>
       </c>
@@ -8255,7 +8266,7 @@
       <c r="E74" s="11"/>
     </row>
     <row r="75" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A75" s="52"/>
+      <c r="A75" s="51"/>
       <c r="B75" s="28" t="s">
         <v>68</v>
       </c>
@@ -8264,7 +8275,7 @@
       <c r="E75" s="25"/>
     </row>
     <row r="76" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A76" s="52"/>
+      <c r="A76" s="51"/>
       <c r="B76" s="18" t="s">
         <v>6</v>
       </c>
@@ -8279,29 +8290,17 @@
       </c>
     </row>
     <row r="77" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A77" s="53"/>
-      <c r="B77" s="54" t="s">
+      <c r="A77" s="52"/>
+      <c r="B77" s="53" t="s">
         <v>71</v>
       </c>
       <c r="C77" s="47"/>
       <c r="D77" s="47"/>
-      <c r="E77" s="58"/>
+      <c r="E77" s="54"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="19">
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="A69:A77"/>
-    <mergeCell ref="B77:E77"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A56:A64"/>
-    <mergeCell ref="B64:E64"/>
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A30:A38"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A43:A51"/>
-    <mergeCell ref="B51:E51"/>
     <mergeCell ref="A17:A25"/>
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="A1:E1"/>
@@ -8309,6 +8308,18 @@
     <mergeCell ref="A4:A12"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A30:A38"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A43:A51"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A69:A77"/>
+    <mergeCell ref="B77:E77"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A56:A64"/>
+    <mergeCell ref="B64:E64"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -8365,7 +8376,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R10</v>
       </c>
@@ -8383,7 +8394,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -8392,7 +8403,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -8401,14 +8412,14 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
         <v>116</v>
       </c>
@@ -8417,7 +8428,7 @@
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>117</v>
       </c>
@@ -8426,7 +8437,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>118</v>
       </c>
@@ -8435,7 +8446,7 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="115.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
@@ -8450,8 +8461,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
         <v>121</v>
       </c>
       <c r="C12" s="48"/>
@@ -8487,7 +8498,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="128.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R11</v>
       </c>
@@ -8505,7 +8516,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -8514,7 +8525,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -8523,14 +8534,14 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>126</v>
       </c>
@@ -8539,7 +8550,7 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>127</v>
       </c>
@@ -8548,7 +8559,7 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
         <v>128</v>
       </c>
@@ -8557,7 +8568,7 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="82.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
@@ -8572,8 +8583,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
         <v>131</v>
       </c>
       <c r="C25" s="48"/>
@@ -8584,7 +8595,7 @@
     <row r="27" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="28" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A28" s="44" t="s">
-        <v>385</v>
+        <v>376</v>
       </c>
       <c r="B28" s="45"/>
       <c r="C28" s="45"/>
@@ -8609,7 +8620,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="128.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v>R12</v>
       </c>
@@ -8617,17 +8628,17 @@
         <v>46</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>386</v>
+        <v>377</v>
       </c>
       <c r="D30" s="6" t="s">
-        <v>387</v>
+        <v>378</v>
       </c>
       <c r="E30" s="7" t="s">
-        <v>388</v>
+        <v>379</v>
       </c>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -8636,7 +8647,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -8645,57 +8656,57 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
-        <v>389</v>
+        <v>380</v>
       </c>
       <c r="C34" s="10"/>
       <c r="D34" s="10"/>
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
-        <v>390</v>
+        <v>381</v>
       </c>
       <c r="C35" s="10"/>
       <c r="D35" s="10"/>
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
-        <v>391</v>
+        <v>382</v>
       </c>
       <c r="C36" s="24"/>
       <c r="D36" s="24"/>
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C37" s="19" t="s">
-        <v>392</v>
+        <v>383</v>
       </c>
       <c r="D37" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E37" s="21" t="s">
-        <v>393</v>
+        <v>384</v>
       </c>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>71</v>
       </c>
       <c r="C38" s="48"/>
@@ -8731,7 +8742,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="153.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="51" t="str">
+      <c r="A43" s="50" t="str">
         <f>LEFT(A41,3)</f>
         <v>R13</v>
       </c>
@@ -8749,7 +8760,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="52"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="23"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -8758,7 +8769,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="52"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="29" t="s">
         <v>8</v>
       </c>
@@ -8767,14 +8778,14 @@
       <c r="E45" s="11"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="52"/>
+      <c r="A46" s="51"/>
       <c r="B46" s="22"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="11"/>
     </row>
     <row r="47" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A47" s="52"/>
+      <c r="A47" s="51"/>
       <c r="B47" s="26" t="s">
         <v>136</v>
       </c>
@@ -8783,7 +8794,7 @@
       <c r="E47" s="11"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="52"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="27" t="s">
         <v>137</v>
       </c>
@@ -8792,7 +8803,7 @@
       <c r="E48" s="11"/>
     </row>
     <row r="49" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="52"/>
+      <c r="A49" s="51"/>
       <c r="B49" s="28" t="s">
         <v>138</v>
       </c>
@@ -8801,7 +8812,7 @@
       <c r="E49" s="25"/>
     </row>
     <row r="50" spans="1:5" ht="86.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="52"/>
+      <c r="A50" s="51"/>
       <c r="B50" s="18" t="s">
         <v>6</v>
       </c>
@@ -8816,8 +8827,8 @@
       </c>
     </row>
     <row r="51" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="53"/>
-      <c r="B51" s="54" t="s">
+      <c r="A51" s="52"/>
+      <c r="B51" s="53" t="s">
         <v>141</v>
       </c>
       <c r="C51" s="48"/>
@@ -8828,11 +8839,6 @@
     <row r="53" spans="1:5" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A4:A12"/>
-    <mergeCell ref="B12:E12"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A15:E15"/>
     <mergeCell ref="A41:E41"/>
     <mergeCell ref="A43:A51"/>
     <mergeCell ref="B51:E51"/>
@@ -8841,6 +8847,11 @@
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A30:A38"/>
     <mergeCell ref="B38:E38"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A4:A12"/>
+    <mergeCell ref="B12:E12"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A15:E15"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -8897,7 +8908,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="128.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R14</v>
       </c>
@@ -8915,7 +8926,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -8924,7 +8935,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -8933,14 +8944,14 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
         <v>147</v>
       </c>
@@ -8949,7 +8960,7 @@
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>148</v>
       </c>
@@ -8958,7 +8969,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>149</v>
       </c>
@@ -8967,7 +8978,7 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
@@ -8982,8 +8993,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
         <v>141</v>
       </c>
       <c r="C12" s="48"/>
@@ -8994,7 +9005,7 @@
     <row r="14" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="44" t="s">
-        <v>394</v>
+        <v>385</v>
       </c>
       <c r="B15" s="45"/>
       <c r="C15" s="45"/>
@@ -9019,7 +9030,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="146.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R15</v>
       </c>
@@ -9027,17 +9038,17 @@
         <v>46</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>395</v>
+        <v>386</v>
       </c>
       <c r="D17" s="6" t="s">
-        <v>396</v>
+        <v>387</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>397</v>
+        <v>388</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -9046,7 +9057,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -9055,23 +9066,23 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="51" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
-        <v>398</v>
+        <v>389</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>152</v>
       </c>
@@ -9080,33 +9091,33 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
-        <v>399</v>
+        <v>390</v>
       </c>
       <c r="C23" s="24"/>
       <c r="D23" s="24"/>
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>400</v>
+        <v>391</v>
       </c>
       <c r="D24" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>401</v>
+        <v>392</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
-        <v>402</v>
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
+        <v>393</v>
       </c>
       <c r="C25" s="48"/>
       <c r="D25" s="48"/>
@@ -9141,7 +9152,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="179.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v>R16</v>
       </c>
@@ -9159,7 +9170,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -9168,7 +9179,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -9177,14 +9188,14 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
         <v>157</v>
       </c>
@@ -9193,7 +9204,7 @@
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
         <v>158</v>
       </c>
@@ -9202,7 +9213,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
         <v>159</v>
       </c>
@@ -9211,7 +9222,7 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="102.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
@@ -9226,8 +9237,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>162</v>
       </c>
       <c r="C38" s="48"/>
@@ -9305,7 +9316,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="102.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R17</v>
       </c>
@@ -9323,7 +9334,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -9332,7 +9343,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -9341,14 +9352,14 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
         <v>168</v>
       </c>
@@ -9357,7 +9368,7 @@
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>169</v>
       </c>
@@ -9366,7 +9377,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>170</v>
       </c>
@@ -9375,7 +9386,7 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
@@ -9390,8 +9401,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
         <v>54</v>
       </c>
       <c r="C12" s="48"/>
@@ -9427,7 +9438,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R18</v>
       </c>
@@ -9445,7 +9456,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -9454,7 +9465,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -9463,14 +9474,14 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>177</v>
       </c>
@@ -9479,7 +9490,7 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>178</v>
       </c>
@@ -9488,7 +9499,7 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
         <v>179</v>
       </c>
@@ -9497,7 +9508,7 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
@@ -9512,8 +9523,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
         <v>182</v>
       </c>
       <c r="C25" s="48"/>
@@ -9549,7 +9560,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="171.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v>R19</v>
       </c>
@@ -9567,7 +9578,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -9576,7 +9587,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -9585,14 +9596,14 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
         <v>187</v>
       </c>
@@ -9601,7 +9612,7 @@
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
         <v>188</v>
       </c>
@@ -9610,7 +9621,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
         <v>189</v>
       </c>
@@ -9619,7 +9630,7 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
@@ -9634,8 +9645,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>192</v>
       </c>
       <c r="C38" s="48"/>
@@ -9713,7 +9724,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="128.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R20</v>
       </c>
@@ -9727,11 +9738,11 @@
         <v>196</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>403</v>
+        <v>394</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -9740,7 +9751,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -9749,23 +9760,23 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
-        <v>404</v>
+        <v>395</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>197</v>
       </c>
@@ -9774,7 +9785,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>198</v>
       </c>
@@ -9783,24 +9794,24 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="77.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>405</v>
+        <v>396</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>406</v>
+        <v>397</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
-        <v>407</v>
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
+        <v>398</v>
       </c>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -9810,7 +9821,7 @@
     <row r="14" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25"/>
     <row r="15" spans="1:5" ht="16.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A15" s="44" t="s">
-        <v>408</v>
+        <v>399</v>
       </c>
       <c r="B15" s="45"/>
       <c r="C15" s="45"/>
@@ -9835,7 +9846,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="153.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R21</v>
       </c>
@@ -9849,11 +9860,11 @@
         <v>200</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>409</v>
+        <v>400</v>
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -9862,7 +9873,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -9871,23 +9882,23 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
-        <v>410</v>
+        <v>401</v>
       </c>
       <c r="C21" s="10"/>
       <c r="D21" s="10"/>
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>201</v>
       </c>
@@ -9896,33 +9907,33 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
-        <v>411</v>
+        <v>402</v>
       </c>
       <c r="C23" s="24"/>
       <c r="D23" s="24"/>
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C24" s="19" t="s">
-        <v>412</v>
+        <v>403</v>
       </c>
       <c r="D24" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E24" s="21" t="s">
-        <v>413</v>
+        <v>404</v>
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
-        <v>414</v>
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
+        <v>405</v>
       </c>
       <c r="C25" s="48"/>
       <c r="D25" s="48"/>
@@ -9957,7 +9968,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="153.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v>R22</v>
       </c>
@@ -9975,7 +9986,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -9984,7 +9995,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -9993,14 +10004,14 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
         <v>206</v>
       </c>
@@ -10009,7 +10020,7 @@
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
         <v>207</v>
       </c>
@@ -10018,7 +10029,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
         <v>208</v>
       </c>
@@ -10027,7 +10038,7 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
@@ -10042,8 +10053,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>211</v>
       </c>
       <c r="C38" s="48"/>
@@ -10079,7 +10090,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="156" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="51" t="str">
+      <c r="A43" s="50" t="str">
         <f>LEFT(A41,3)</f>
         <v>R23</v>
       </c>
@@ -10097,7 +10108,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="52"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="23"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -10106,7 +10117,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="52"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="29" t="s">
         <v>8</v>
       </c>
@@ -10115,14 +10126,14 @@
       <c r="E45" s="11"/>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A46" s="52"/>
+      <c r="A46" s="51"/>
       <c r="B46" s="22"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="11"/>
     </row>
     <row r="47" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A47" s="52"/>
+      <c r="A47" s="51"/>
       <c r="B47" s="26" t="s">
         <v>216</v>
       </c>
@@ -10131,7 +10142,7 @@
       <c r="E47" s="11"/>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A48" s="52"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="27" t="s">
         <v>217</v>
       </c>
@@ -10140,7 +10151,7 @@
       <c r="E48" s="11"/>
     </row>
     <row r="49" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="52"/>
+      <c r="A49" s="51"/>
       <c r="B49" s="28" t="s">
         <v>218</v>
       </c>
@@ -10149,7 +10160,7 @@
       <c r="E49" s="25"/>
     </row>
     <row r="50" spans="1:5" ht="94.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="52"/>
+      <c r="A50" s="51"/>
       <c r="B50" s="18" t="s">
         <v>6</v>
       </c>
@@ -10164,8 +10175,8 @@
       </c>
     </row>
     <row r="51" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="53"/>
-      <c r="B51" s="54" t="s">
+      <c r="A51" s="52"/>
+      <c r="B51" s="53" t="s">
         <v>221</v>
       </c>
       <c r="C51" s="48"/>
@@ -10201,7 +10212,7 @@
       </c>
     </row>
     <row r="56" spans="1:5" ht="128.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A56" s="51" t="str">
+      <c r="A56" s="50" t="str">
         <f>LEFT(A54,3)</f>
         <v>R24</v>
       </c>
@@ -10219,7 +10230,7 @@
       </c>
     </row>
     <row r="57" spans="1:5" ht="13.5" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A57" s="52"/>
+      <c r="A57" s="51"/>
       <c r="B57" s="23"/>
       <c r="C57" s="8"/>
       <c r="D57" s="8"/>
@@ -10228,7 +10239,7 @@
       </c>
     </row>
     <row r="58" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="52"/>
+      <c r="A58" s="51"/>
       <c r="B58" s="29" t="s">
         <v>8</v>
       </c>
@@ -10237,14 +10248,14 @@
       <c r="E58" s="11"/>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A59" s="52"/>
+      <c r="A59" s="51"/>
       <c r="B59" s="22"/>
       <c r="C59" s="10"/>
       <c r="D59" s="10"/>
       <c r="E59" s="11"/>
     </row>
     <row r="60" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A60" s="52"/>
+      <c r="A60" s="51"/>
       <c r="B60" s="26" t="s">
         <v>226</v>
       </c>
@@ -10253,7 +10264,7 @@
       <c r="E60" s="11"/>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A61" s="52"/>
+      <c r="A61" s="51"/>
       <c r="B61" s="27" t="s">
         <v>227</v>
       </c>
@@ -10262,7 +10273,7 @@
       <c r="E61" s="11"/>
     </row>
     <row r="62" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="52"/>
+      <c r="A62" s="51"/>
       <c r="B62" s="28" t="s">
         <v>228</v>
       </c>
@@ -10271,7 +10282,7 @@
       <c r="E62" s="25"/>
     </row>
     <row r="63" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A63" s="52"/>
+      <c r="A63" s="51"/>
       <c r="B63" s="18" t="s">
         <v>6</v>
       </c>
@@ -10286,8 +10297,8 @@
       </c>
     </row>
     <row r="64" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A64" s="53"/>
-      <c r="B64" s="54" t="s">
+      <c r="A64" s="52"/>
+      <c r="B64" s="53" t="s">
         <v>231</v>
       </c>
       <c r="C64" s="48"/>
@@ -10323,7 +10334,7 @@
       </c>
     </row>
     <row r="69" spans="1:5" customFormat="1" ht="122.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A69" s="51" t="str">
+      <c r="A69" s="50" t="str">
         <f>LEFT(A67,3)</f>
         <v>R25</v>
       </c>
@@ -10341,7 +10352,7 @@
       </c>
     </row>
     <row r="70" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A70" s="52"/>
+      <c r="A70" s="51"/>
       <c r="B70" s="23"/>
       <c r="C70" s="8"/>
       <c r="D70" s="8"/>
@@ -10350,7 +10361,7 @@
       </c>
     </row>
     <row r="71" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A71" s="52"/>
+      <c r="A71" s="51"/>
       <c r="B71" s="29" t="s">
         <v>8</v>
       </c>
@@ -10359,14 +10370,14 @@
       <c r="E71" s="11"/>
     </row>
     <row r="72" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A72" s="52"/>
+      <c r="A72" s="51"/>
       <c r="B72" s="22"/>
       <c r="C72" s="10"/>
       <c r="D72" s="10"/>
       <c r="E72" s="11"/>
     </row>
     <row r="73" spans="1:5" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A73" s="52"/>
+      <c r="A73" s="51"/>
       <c r="B73" s="26" t="s">
         <v>236</v>
       </c>
@@ -10375,7 +10386,7 @@
       <c r="E73" s="11"/>
     </row>
     <row r="74" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A74" s="52"/>
+      <c r="A74" s="51"/>
       <c r="B74" s="27" t="s">
         <v>237</v>
       </c>
@@ -10384,7 +10395,7 @@
       <c r="E74" s="11"/>
     </row>
     <row r="75" spans="1:5" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A75" s="52"/>
+      <c r="A75" s="51"/>
       <c r="B75" s="28" t="s">
         <v>238</v>
       </c>
@@ -10393,7 +10404,7 @@
       <c r="E75" s="25"/>
     </row>
     <row r="76" spans="1:5" customFormat="1" ht="81.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A76" s="52"/>
+      <c r="A76" s="51"/>
       <c r="B76" s="18" t="s">
         <v>6</v>
       </c>
@@ -10408,8 +10419,8 @@
       </c>
     </row>
     <row r="77" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A77" s="53"/>
-      <c r="B77" s="54" t="s">
+      <c r="A77" s="52"/>
+      <c r="B77" s="53" t="s">
         <v>241</v>
       </c>
       <c r="C77" s="48"/>
@@ -10445,7 +10456,7 @@
       </c>
     </row>
     <row r="82" spans="1:5" customFormat="1" ht="217.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A82" s="51" t="str">
+      <c r="A82" s="50" t="str">
         <f>LEFT(A80,3)</f>
         <v>R26</v>
       </c>
@@ -10463,7 +10474,7 @@
       </c>
     </row>
     <row r="83" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A83" s="52"/>
+      <c r="A83" s="51"/>
       <c r="B83" s="23"/>
       <c r="C83" s="8"/>
       <c r="D83" s="8"/>
@@ -10472,7 +10483,7 @@
       </c>
     </row>
     <row r="84" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A84" s="52"/>
+      <c r="A84" s="51"/>
       <c r="B84" s="29" t="s">
         <v>8</v>
       </c>
@@ -10481,14 +10492,14 @@
       <c r="E84" s="11"/>
     </row>
     <row r="85" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A85" s="52"/>
+      <c r="A85" s="51"/>
       <c r="B85" s="22"/>
       <c r="C85" s="10"/>
       <c r="D85" s="10"/>
       <c r="E85" s="11"/>
     </row>
     <row r="86" spans="1:5" customFormat="1" ht="38.25" x14ac:dyDescent="0.25">
-      <c r="A86" s="52"/>
+      <c r="A86" s="51"/>
       <c r="B86" s="26" t="s">
         <v>246</v>
       </c>
@@ -10497,7 +10508,7 @@
       <c r="E86" s="11"/>
     </row>
     <row r="87" spans="1:5" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A87" s="52"/>
+      <c r="A87" s="51"/>
       <c r="B87" s="27" t="s">
         <v>247</v>
       </c>
@@ -10506,7 +10517,7 @@
       <c r="E87" s="11"/>
     </row>
     <row r="88" spans="1:5" customFormat="1" ht="26.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A88" s="52"/>
+      <c r="A88" s="51"/>
       <c r="B88" s="28" t="s">
         <v>248</v>
       </c>
@@ -10515,7 +10526,7 @@
       <c r="E88" s="25"/>
     </row>
     <row r="89" spans="1:5" customFormat="1" ht="77.25" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A89" s="52"/>
+      <c r="A89" s="51"/>
       <c r="B89" s="18" t="s">
         <v>6</v>
       </c>
@@ -10530,8 +10541,8 @@
       </c>
     </row>
     <row r="90" spans="1:5" customFormat="1" ht="12.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="53"/>
-      <c r="B90" s="54" t="s">
+      <c r="A90" s="52"/>
+      <c r="B90" s="53" t="s">
         <v>251</v>
       </c>
       <c r="C90" s="48"/>
@@ -10542,17 +10553,6 @@
     <row r="92" spans="1:5" ht="12.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="22">
-    <mergeCell ref="A67:E67"/>
-    <mergeCell ref="A69:A77"/>
-    <mergeCell ref="B77:E77"/>
-    <mergeCell ref="A80:E80"/>
-    <mergeCell ref="A82:A90"/>
-    <mergeCell ref="B90:E90"/>
-    <mergeCell ref="A43:A51"/>
-    <mergeCell ref="B51:E51"/>
-    <mergeCell ref="A54:E54"/>
-    <mergeCell ref="A56:A64"/>
-    <mergeCell ref="B64:E64"/>
     <mergeCell ref="A28:E28"/>
     <mergeCell ref="A30:A38"/>
     <mergeCell ref="B38:E38"/>
@@ -10564,6 +10564,17 @@
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A17:A25"/>
     <mergeCell ref="B25:E25"/>
+    <mergeCell ref="A43:A51"/>
+    <mergeCell ref="B51:E51"/>
+    <mergeCell ref="A54:E54"/>
+    <mergeCell ref="A56:A64"/>
+    <mergeCell ref="B64:E64"/>
+    <mergeCell ref="A67:E67"/>
+    <mergeCell ref="A69:A77"/>
+    <mergeCell ref="B77:E77"/>
+    <mergeCell ref="A80:E80"/>
+    <mergeCell ref="A82:A90"/>
+    <mergeCell ref="B90:E90"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -10620,7 +10631,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="115.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R27</v>
       </c>
@@ -10638,7 +10649,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -10647,7 +10658,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -10656,14 +10667,14 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
         <v>258</v>
       </c>
@@ -10672,7 +10683,7 @@
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>259</v>
       </c>
@@ -10681,7 +10692,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>260</v>
       </c>
@@ -10690,7 +10701,7 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
@@ -10705,8 +10716,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
         <v>263</v>
       </c>
       <c r="C12" s="48"/>
@@ -10742,7 +10753,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="166.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R28</v>
       </c>
@@ -10760,7 +10771,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -10769,7 +10780,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -10778,14 +10789,14 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>268</v>
       </c>
@@ -10794,7 +10805,7 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>269</v>
       </c>
@@ -10803,7 +10814,7 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
         <v>270</v>
       </c>
@@ -10812,7 +10823,7 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
@@ -10827,8 +10838,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
         <v>273</v>
       </c>
       <c r="C25" s="48"/>
@@ -10864,7 +10875,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="115.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v>R29</v>
       </c>
@@ -10882,7 +10893,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -10891,7 +10902,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -10900,14 +10911,14 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
         <v>278</v>
       </c>
@@ -10916,7 +10927,7 @@
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
         <v>279</v>
       </c>
@@ -10925,7 +10936,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
         <v>280</v>
       </c>
@@ -10934,7 +10945,7 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
@@ -10949,8 +10960,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>283</v>
       </c>
       <c r="C38" s="48"/>
@@ -11027,7 +11038,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="90" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R30</v>
       </c>
@@ -11045,7 +11056,7 @@
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -11054,7 +11065,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -11063,14 +11074,14 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
         <v>289</v>
       </c>
@@ -11079,7 +11090,7 @@
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>290</v>
       </c>
@@ -11088,7 +11099,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>291</v>
       </c>
@@ -11097,7 +11108,7 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
@@ -11112,8 +11123,8 @@
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
         <v>294</v>
       </c>
       <c r="C12" s="48"/>
@@ -11149,7 +11160,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="115.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R31</v>
       </c>
@@ -11167,7 +11178,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -11176,7 +11187,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -11185,14 +11196,14 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>298</v>
       </c>
@@ -11201,7 +11212,7 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>299</v>
       </c>
@@ -11210,7 +11221,7 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
         <v>300</v>
       </c>
@@ -11219,7 +11230,7 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="51.75" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
@@ -11234,8 +11245,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
         <v>303</v>
       </c>
       <c r="C25" s="48"/>
@@ -11271,7 +11282,7 @@
       </c>
     </row>
     <row r="30" spans="1:5" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A30" s="51" t="str">
+      <c r="A30" s="50" t="str">
         <f>LEFT(A28,3)</f>
         <v>R32</v>
       </c>
@@ -11289,7 +11300,7 @@
       </c>
     </row>
     <row r="31" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A31" s="52"/>
+      <c r="A31" s="51"/>
       <c r="B31" s="23"/>
       <c r="C31" s="8"/>
       <c r="D31" s="8"/>
@@ -11298,7 +11309,7 @@
       </c>
     </row>
     <row r="32" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A32" s="52"/>
+      <c r="A32" s="51"/>
       <c r="B32" s="29" t="s">
         <v>8</v>
       </c>
@@ -11307,14 +11318,14 @@
       <c r="E32" s="11"/>
     </row>
     <row r="33" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A33" s="52"/>
+      <c r="A33" s="51"/>
       <c r="B33" s="22"/>
       <c r="C33" s="10"/>
       <c r="D33" s="10"/>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A34" s="52"/>
+      <c r="A34" s="51"/>
       <c r="B34" s="26" t="s">
         <v>309</v>
       </c>
@@ -11323,7 +11334,7 @@
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A35" s="52"/>
+      <c r="A35" s="51"/>
       <c r="B35" s="27" t="s">
         <v>310</v>
       </c>
@@ -11332,7 +11343,7 @@
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="52"/>
+      <c r="A36" s="51"/>
       <c r="B36" s="28" t="s">
         <v>311</v>
       </c>
@@ -11341,7 +11352,7 @@
       <c r="E36" s="25"/>
     </row>
     <row r="37" spans="1:5" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="52"/>
+      <c r="A37" s="51"/>
       <c r="B37" s="18" t="s">
         <v>6</v>
       </c>
@@ -11356,8 +11367,8 @@
       </c>
     </row>
     <row r="38" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="53"/>
-      <c r="B38" s="54" t="s">
+      <c r="A38" s="52"/>
+      <c r="B38" s="53" t="s">
         <v>314</v>
       </c>
       <c r="C38" s="48"/>
@@ -11393,7 +11404,7 @@
       </c>
     </row>
     <row r="43" spans="1:5" ht="141" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="51" t="str">
+      <c r="A43" s="50" t="str">
         <f>LEFT(A41,3)</f>
         <v>R33</v>
       </c>
@@ -11411,7 +11422,7 @@
       </c>
     </row>
     <row r="44" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A44" s="52"/>
+      <c r="A44" s="51"/>
       <c r="B44" s="23"/>
       <c r="C44" s="8"/>
       <c r="D44" s="8"/>
@@ -11420,7 +11431,7 @@
       </c>
     </row>
     <row r="45" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A45" s="52"/>
+      <c r="A45" s="51"/>
       <c r="B45" s="29" t="s">
         <v>8</v>
       </c>
@@ -11429,14 +11440,14 @@
       <c r="E45" s="11"/>
     </row>
     <row r="46" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A46" s="52"/>
+      <c r="A46" s="51"/>
       <c r="B46" s="22"/>
       <c r="C46" s="10"/>
       <c r="D46" s="10"/>
       <c r="E46" s="11"/>
     </row>
     <row r="47" spans="1:5" ht="51" x14ac:dyDescent="0.2">
-      <c r="A47" s="52"/>
+      <c r="A47" s="51"/>
       <c r="B47" s="26" t="s">
         <v>319</v>
       </c>
@@ -11445,7 +11456,7 @@
       <c r="E47" s="11"/>
     </row>
     <row r="48" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="52"/>
+      <c r="A48" s="51"/>
       <c r="B48" s="27" t="s">
         <v>320</v>
       </c>
@@ -11454,7 +11465,7 @@
       <c r="E48" s="11"/>
     </row>
     <row r="49" spans="1:5" ht="26.25" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="52"/>
+      <c r="A49" s="51"/>
       <c r="B49" s="28" t="s">
         <v>321</v>
       </c>
@@ -11463,7 +11474,7 @@
       <c r="E49" s="25"/>
     </row>
     <row r="50" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="52"/>
+      <c r="A50" s="51"/>
       <c r="B50" s="18" t="s">
         <v>6</v>
       </c>
@@ -11478,8 +11489,8 @@
       </c>
     </row>
     <row r="51" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="53"/>
-      <c r="B51" s="54" t="s">
+      <c r="A51" s="52"/>
+      <c r="B51" s="53" t="s">
         <v>324</v>
       </c>
       <c r="C51" s="48"/>
@@ -11492,12 +11503,6 @@
     <row r="55" spans="1:5" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="A28:E28"/>
-    <mergeCell ref="A30:A38"/>
-    <mergeCell ref="B38:E38"/>
-    <mergeCell ref="A41:E41"/>
-    <mergeCell ref="A43:A51"/>
-    <mergeCell ref="B51:E51"/>
     <mergeCell ref="A17:A25"/>
     <mergeCell ref="B25:E25"/>
     <mergeCell ref="A1:E1"/>
@@ -11505,6 +11510,12 @@
     <mergeCell ref="A4:A12"/>
     <mergeCell ref="B12:E12"/>
     <mergeCell ref="A15:E15"/>
+    <mergeCell ref="A28:E28"/>
+    <mergeCell ref="A30:A38"/>
+    <mergeCell ref="B38:E38"/>
+    <mergeCell ref="A41:E41"/>
+    <mergeCell ref="A43:A51"/>
+    <mergeCell ref="B51:E51"/>
   </mergeCells>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="5" orientation="landscape" r:id="rId1"/>
@@ -11561,7 +11572,7 @@
       </c>
     </row>
     <row r="4" spans="1:5" ht="121.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="51" t="str">
+      <c r="A4" s="50" t="str">
         <f>LEFT(A2,3)</f>
         <v>R34</v>
       </c>
@@ -11572,14 +11583,14 @@
         <v>327</v>
       </c>
       <c r="D4" s="6" t="s">
-        <v>415</v>
+        <v>406</v>
       </c>
       <c r="E4" s="7" t="s">
-        <v>416</v>
+        <v>407</v>
       </c>
     </row>
     <row r="5" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="52"/>
+      <c r="A5" s="51"/>
       <c r="B5" s="23"/>
       <c r="C5" s="8"/>
       <c r="D5" s="8"/>
@@ -11588,7 +11599,7 @@
       </c>
     </row>
     <row r="6" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="52"/>
+      <c r="A6" s="51"/>
       <c r="B6" s="29" t="s">
         <v>8</v>
       </c>
@@ -11597,23 +11608,23 @@
       <c r="E6" s="11"/>
     </row>
     <row r="7" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A7" s="52"/>
+      <c r="A7" s="51"/>
       <c r="B7" s="22"/>
       <c r="C7" s="10"/>
       <c r="D7" s="10"/>
       <c r="E7" s="11"/>
     </row>
     <row r="8" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A8" s="52"/>
+      <c r="A8" s="51"/>
       <c r="B8" s="26" t="s">
-        <v>417</v>
+        <v>408</v>
       </c>
       <c r="C8" s="10"/>
       <c r="D8" s="10"/>
       <c r="E8" s="11"/>
     </row>
     <row r="9" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="52"/>
+      <c r="A9" s="51"/>
       <c r="B9" s="27" t="s">
         <v>328</v>
       </c>
@@ -11622,7 +11633,7 @@
       <c r="E9" s="11"/>
     </row>
     <row r="10" spans="1:5" ht="26.25" hidden="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="52"/>
+      <c r="A10" s="51"/>
       <c r="B10" s="28" t="s">
         <v>329</v>
       </c>
@@ -11631,24 +11642,24 @@
       <c r="E10" s="25"/>
     </row>
     <row r="11" spans="1:5" ht="64.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A11" s="52"/>
+      <c r="A11" s="51"/>
       <c r="B11" s="18" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="19" t="s">
-        <v>418</v>
+        <v>409</v>
       </c>
       <c r="D11" s="20" t="s">
         <v>7</v>
       </c>
       <c r="E11" s="21" t="s">
-        <v>419</v>
+        <v>410</v>
       </c>
     </row>
     <row r="12" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="53"/>
-      <c r="B12" s="54" t="s">
-        <v>420</v>
+      <c r="A12" s="52"/>
+      <c r="B12" s="53" t="s">
+        <v>411</v>
       </c>
       <c r="C12" s="48"/>
       <c r="D12" s="48"/>
@@ -11683,7 +11694,7 @@
       </c>
     </row>
     <row r="17" spans="1:5" ht="156" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="51" t="str">
+      <c r="A17" s="50" t="str">
         <f>LEFT(A15,3)</f>
         <v>R35</v>
       </c>
@@ -11701,7 +11712,7 @@
       </c>
     </row>
     <row r="18" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="52"/>
+      <c r="A18" s="51"/>
       <c r="B18" s="23"/>
       <c r="C18" s="8"/>
       <c r="D18" s="8"/>
@@ -11710,7 +11721,7 @@
       </c>
     </row>
     <row r="19" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="52"/>
+      <c r="A19" s="51"/>
       <c r="B19" s="29" t="s">
         <v>8</v>
       </c>
@@ -11719,14 +11730,14 @@
       <c r="E19" s="11"/>
     </row>
     <row r="20" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A20" s="52"/>
+      <c r="A20" s="51"/>
       <c r="B20" s="22"/>
       <c r="C20" s="10"/>
       <c r="D20" s="10"/>
       <c r="E20" s="11"/>
     </row>
     <row r="21" spans="1:5" ht="38.25" x14ac:dyDescent="0.2">
-      <c r="A21" s="52"/>
+      <c r="A21" s="51"/>
       <c r="B21" s="26" t="s">
         <v>334</v>
       </c>
@@ -11735,7 +11746,7 @@
       <c r="E21" s="11"/>
     </row>
     <row r="22" spans="1:5" ht="12.75" x14ac:dyDescent="0.2">
-      <c r="A22" s="52"/>
+      <c r="A22" s="51"/>
       <c r="B22" s="27" t="s">
         <v>335</v>
       </c>
@@ -11744,7 +11755,7 @@
       <c r="E22" s="11"/>
     </row>
     <row r="23" spans="1:5" ht="26.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="52"/>
+      <c r="A23" s="51"/>
       <c r="B23" s="28" t="s">
         <v>336</v>
       </c>
@@ -11753,7 +11764,7 @@
       <c r="E23" s="25"/>
     </row>
     <row r="24" spans="1:5" ht="77.25" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A24" s="52"/>
+      <c r="A24" s="51"/>
       <c r="B24" s="18" t="s">
         <v>6</v>
       </c>
@@ -11768,8 +11779,8 @@
       </c>
     </row>
     <row r="25" spans="1:5" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="53"/>
-      <c r="B25" s="54" t="s">
+      <c r="A25" s="52"/>
+      <c r="B25" s="53" t="s">
         <v>339</v>
       </c>
       <c r="C25" s="48"/>

</xml_diff>